<commit_message>
Authors, affiliations and ORCID iDs in metadata, licence, tables and preprint
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019utTifuXP1XtTYCS5CjKaD
</commit_message>
<xml_diff>
--- a/results/extra/supplementary_table2_sequence_evidence.xlsx
+++ b/results/extra/supplementary_table2_sequence_evidence.xlsx
@@ -491,7 +491,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Afzoon &amp; Biswal, "Calibrated genome scans find recurrent gene loss in marine and subterranean mammals". Column definitions are in the sheet "Column definitions".</t>
+          <t>Konhar, Afzoon &amp; Biswal, "Calibrated genome scans find recurrent gene loss in marine and subterranean mammals". Column definitions are in the sheet "Column definitions".</t>
         </is>
       </c>
     </row>
@@ -4073,7 +4073,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Afzoon &amp; Biswal, "Calibrated genome scans find recurrent gene loss in marine and subterranean mammals". Column definitions are in the sheet "Column definitions".</t>
+          <t>Konhar, Afzoon &amp; Biswal, "Calibrated genome scans find recurrent gene loss in marine and subterranean mammals". Column definitions are in the sheet "Column definitions".</t>
         </is>
       </c>
     </row>

</xml_diff>